<commit_message>
Daily EOD data and reports for 2026-08-11
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260811.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260811.xlsx
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.345</v>
+        <v>2.335</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.005</v>
+        <v>-0.015</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.21%</t>
+          <t>-0.64%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>164150</v>
+        <v>163450</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-350</v>
+        <v>-1050</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>64.29000000000001</v>
+        <v>64.27</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.21%</t>
+          <t>1.18%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>711368.85</v>
+        <v>711147.55</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>8520.049999999999</v>
+        <v>8298.75</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>174</v>
+        <v>173.9</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.27</v>
+        <v>-0.37</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.15%</t>
+          <t>-0.21%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.915</v>
+        <v>0.92</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.01</v>
+        <v>0.015</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>1.66%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9150</v>
+        <v>9200</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>138.64</v>
+        <v>138.34</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>4.17</v>
+        <v>3.87</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.10%</t>
+          <t>2.88%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>554560</v>
+        <v>553360</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>16680</v>
+        <v>15480</v>
       </c>
     </row>
     <row r="12">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.105</v>
+        <v>0.1</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.008</v>
+        <v>0.003</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.25%</t>
+          <t>3.09%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>988.26</v>
+        <v>941.2</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>75.3</v>
+        <v>28.24</v>
       </c>
     </row>
     <row r="15">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>35.6</v>
+        <v>35.55</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.28%</t>
+          <t>-0.42%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.91</v>
+        <v>32.94</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.12</v>
+        <v>1.15</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3.52%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42388.08</v>
+        <v>42426.72</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1442.56</v>
+        <v>1481.2</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1803095.73</v>
+        <v>1801016.01</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>28010.54</v>
+        <v>25930.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>